<commit_message>
Auto-seed Dhiraj and Praveen and embed Google Sheets sync in Streamlit Cloud
</commit_message>
<xml_diff>
--- a/Student_Academic_Progression_Data.xlsx
+++ b/Student_Academic_Progression_Data.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -656,6 +656,144 @@
       <c r="J5" t="inlineStr">
         <is>
           <t>2026-10-27 05:46:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CE-2026-048</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dhiraj suthar</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>gaurishankaryadav896@gmail.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>7420961073</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-10-27 06:21:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CE-2025-99</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Praveen tiwari</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>praveen86@gmail.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>9619561398</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-10-27 06:26:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ECE-2025-31</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Vyomesh Shetty</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>vyomesh79@gmail.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1298763536</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Electrical and Computer Engineering</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-10-27 07:15:58</t>
         </is>
       </c>
     </row>
@@ -670,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -799,6 +937,78 @@
       </c>
       <c r="F5" t="n">
         <v>2020</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CE-2026-048</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>dhiraj suthar</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>75</v>
+      </c>
+      <c r="E6" t="n">
+        <v>67</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CE-2025-99</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Praveen tiwari</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>92</v>
+      </c>
+      <c r="E7" t="n">
+        <v>99</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ECE-2025-31</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Vyomesh Shetty</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>97</v>
+      </c>
+      <c r="E8" t="n">
+        <v>98</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Seed Gaurishankar Yadav and Vyomesh Shetty and update spreadsheet
</commit_message>
<xml_diff>
--- a/Student_Academic_Progression_Data.xlsx
+++ b/Student_Academic_Progression_Data.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -794,6 +794,52 @@
       <c r="J8" t="inlineStr">
         <is>
           <t>2026-10-27 07:15:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CE-2022-001</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Gaurishankar Yadav</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>gaurishankar.yadav@example.edu</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>+91 98765 00001</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-10-27 08:03:47</t>
         </is>
       </c>
     </row>
@@ -808,7 +854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1009,6 +1055,30 @@
       </c>
       <c r="F8" t="n">
         <v>2000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CE-2022-001</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Gaurishankar Yadav</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>92</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2022</v>
       </c>
     </row>
   </sheetData>
@@ -1022,7 +1092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1704,6 +1774,216 @@
       <c r="J16" t="inlineStr">
         <is>
           <t>Gold Medalist / College Valedictorian</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CE-2022-001</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Gaurishankar Yadav</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2022-2023</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="H17" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Outstanding first semester</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CE-2022-001</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Gaurishankar Yadav</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2022-2023</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H18" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Dean List Honoree</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>10</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CE-2022-001</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Gaurishankar Yadav</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2023-2024</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H19" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>DBMS Subject Topper</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CE-2022-001</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Gaurishankar Yadav</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2023-2024</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="H20" t="n">
+        <v>9.43</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Full-Stack Project Distinction</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>10</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CE-2022-001</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Gaurishankar Yadav</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2024-2025</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H21" t="n">
+        <v>9.44</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>High Academic Progression</t>
         </is>
       </c>
     </row>

</xml_diff>